<commit_message>
scan: seg0 2026-10-06 02:26 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-05.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-05.xlsx
@@ -633,21 +633,21 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>1326</v>
+        <v>1569</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>台化</t>
+          <t>濱川</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>955.5074210307712</v>
+        <v>963.2329512120886</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>71.59999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,13 +658,13 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>59.82798828216806</v>
+        <v>78.29839855836863</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>28.49140989435775</v>
+        <v>59.96617862328991</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.9988176158365332</v>
+        <v>1.923295121208853</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
@@ -676,31 +676,31 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.08605308859099201</v>
+        <v>0.9831704391127448</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>1569</v>
+        <v>1326</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>濱川</t>
+          <t>台化</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>933.2329512120886</v>
+        <v>955.5074210307712</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>68.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,13 +711,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>78.29839855836863</v>
+        <v>59.82798828216806</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>59.96617862328991</v>
+        <v>28.49140989435775</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.923295121208853</v>
+        <v>0.9988176158365332</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
@@ -729,11 +729,11 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.9831704391127448</v>
+        <v>0.08605308859099201</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>

</xml_diff>